<commit_message>
Refactor material files: remove outdated images and HTML templates, add new welcome letter assets for VRIM
</commit_message>
<xml_diff>
--- a/PruebasCorreos.xlsx
+++ b/PruebasCorreos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roberto Monjardin\Desktop\Salud Interactiva\projects\salud-interactiva-mailing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Desktop\FarmaLeal-Mailing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49069602-E045-4DFA-9DD8-D1B0185E0964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F55B03A6-323F-4D0C-9567-518287B86CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-156" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B3DB81C5-9EF5-45C7-8B63-AD43FCE30ABD}"/>
+    <workbookView xWindow="51480" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{B3DB81C5-9EF5-45C7-8B63-AD43FCE30ABD}"/>
   </bookViews>
   <sheets>
     <sheet name="DETALLE" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="37">
   <si>
     <t>UN</t>
   </si>
@@ -114,25 +114,43 @@
     <t>christian.lepe@farmaleal.com.mx</t>
   </si>
   <si>
-    <t>#EMPLEADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE COMPLETO </t>
-  </si>
-  <si>
-    <t>VIGENCIA</t>
-  </si>
-  <si>
-    <t>PRODUCTO</t>
-  </si>
-  <si>
-    <t>01/Feb/2026 al 01/Feb/2027</t>
-  </si>
-  <si>
-    <t>MEDICALLHOME</t>
-  </si>
-  <si>
     <t>rmonjardin@salud-interactiva.com.mx</t>
+  </si>
+  <si>
+    <t>Producto</t>
+  </si>
+  <si>
+    <t>NumeroTarjeta</t>
+  </si>
+  <si>
+    <t>NomCompleto</t>
+  </si>
+  <si>
+    <t>VIG</t>
+  </si>
+  <si>
+    <t>EtiquetaLogistica02</t>
+  </si>
+  <si>
+    <t>EtiquetaLogistica03</t>
+  </si>
+  <si>
+    <t>BLACK VRIM DIGITAL- GENERICO</t>
+  </si>
+  <si>
+    <t>'1122052600028094</t>
+  </si>
+  <si>
+    <t>'14/MAY/2027</t>
+  </si>
+  <si>
+    <t>'1122052600028096</t>
+  </si>
+  <si>
+    <t>Christian Lepe Cruz</t>
+  </si>
+  <si>
+    <t>clepe@salud-interactiva.com.mx</t>
   </si>
 </sst>
 </file>
@@ -142,7 +160,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,12 +203,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -206,22 +218,11 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="4"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -243,7 +244,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1"/>
@@ -258,14 +259,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -891,71 +885,127 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7100985-58AA-4CEE-9961-6E7E20BF57C2}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="37.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="11">
-        <v>36918</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
-        <v>39481</v>
-      </c>
-      <c r="B3" s="10" t="s">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="7" t="s">
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>17</v>
       </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D10" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{4E5296D9-F0BF-42BE-B77C-CD8F32EC79CF}"/>
-    <hyperlink ref="E2" r:id="rId2" display="mailto:rmonjardin@salud-interactiva.com.mx" xr:uid="{53AF5F3A-31C5-4EBF-B8AA-414536053990}"/>
+    <hyperlink ref="F2" r:id="rId1" display="mailto:rmonjardin@salud-interactiva.com.mx" xr:uid="{BE9F2FF6-456F-4E2B-A0C0-BD76E4E06139}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{091242AC-0F01-4ACA-8F19-964AD4F5C500}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{688216C2-7797-4EEC-9184-3CB51A47873F}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{A8FD61FC-4A75-44A7-BEE5-AD712FBB5B75}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add new email templates and images for reembolso benefits; remove obsolete files
</commit_message>
<xml_diff>
--- a/PruebasCorreos.xlsx
+++ b/PruebasCorreos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Desktop\FarmaLeal-Mailing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roberto Monjardin\Desktop\Salud Interactiva\projects\mailing-salud-interactiva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F55B03A6-323F-4D0C-9567-518287B86CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F660EF-B049-4DFE-A1FF-6D9C806321E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{B3DB81C5-9EF5-45C7-8B63-AD43FCE30ABD}"/>
+    <workbookView xWindow="1095" yWindow="3120" windowWidth="17280" windowHeight="8925" activeTab="1" xr2:uid="{B3DB81C5-9EF5-45C7-8B63-AD43FCE30ABD}"/>
   </bookViews>
   <sheets>
     <sheet name="DETALLE" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t>UN</t>
   </si>
@@ -114,43 +114,49 @@
     <t>christian.lepe@farmaleal.com.mx</t>
   </si>
   <si>
+    <t>Número de Empleado</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Paterno</t>
+  </si>
+  <si>
+    <t>Materno</t>
+  </si>
+  <si>
+    <t>correo</t>
+  </si>
+  <si>
+    <t>Roberto Edgar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monjardin </t>
+  </si>
+  <si>
+    <t>Alvarado</t>
+  </si>
+  <si>
     <t>rmonjardin@salud-interactiva.com.mx</t>
   </si>
   <si>
-    <t>Producto</t>
-  </si>
-  <si>
-    <t>NumeroTarjeta</t>
-  </si>
-  <si>
-    <t>NomCompleto</t>
-  </si>
-  <si>
-    <t>VIG</t>
-  </si>
-  <si>
-    <t>EtiquetaLogistica02</t>
-  </si>
-  <si>
-    <t>EtiquetaLogistica03</t>
-  </si>
-  <si>
-    <t>BLACK VRIM DIGITAL- GENERICO</t>
-  </si>
-  <si>
-    <t>'1122052600028094</t>
-  </si>
-  <si>
-    <t>'14/MAY/2027</t>
-  </si>
-  <si>
-    <t>'1122052600028096</t>
-  </si>
-  <si>
-    <t>Christian Lepe Cruz</t>
-  </si>
-  <si>
-    <t>clepe@salud-interactiva.com.mx</t>
+    <t xml:space="preserve">Maricela </t>
+  </si>
+  <si>
+    <t>Castro</t>
+  </si>
+  <si>
+    <t>mcastro@salud-interactiva.com.mx</t>
+  </si>
+  <si>
+    <t>lhernandez@salud-interactiva.com.mx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liliana </t>
+  </si>
+  <si>
+    <t>Hernández</t>
   </si>
 </sst>
 </file>
@@ -160,7 +166,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -203,6 +209,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -218,20 +230,11 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -244,7 +247,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1"/>
@@ -259,9 +262,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -885,9 +893,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7100985-58AA-4CEE-9961-6E7E20BF57C2}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
     <col min="2" max="2" width="37.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -895,117 +904,76 @@
     <col min="6" max="6" width="41.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="11">
+        <v>207027233</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="F1" t="s">
+      <c r="C2" s="10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="D2" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="11">
+        <v>200423223</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="10" t="s">
+      <c r="D3" s="10"/>
+      <c r="E3" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" s="7" t="s">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="11">
+        <v>200423223</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D10" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="mailto:rmonjardin@salud-interactiva.com.mx" xr:uid="{BE9F2FF6-456F-4E2B-A0C0-BD76E4E06139}"/>
-    <hyperlink ref="F3" r:id="rId2" xr:uid="{091242AC-0F01-4ACA-8F19-964AD4F5C500}"/>
-    <hyperlink ref="F4" r:id="rId3" xr:uid="{688216C2-7797-4EEC-9184-3CB51A47873F}"/>
-    <hyperlink ref="F5" r:id="rId4" xr:uid="{A8FD61FC-4A75-44A7-BEE5-AD712FBB5B75}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{44F4011C-3569-455B-8910-D4651CB76C8C}"/>
+    <hyperlink ref="E3" r:id="rId2" display="mailto:mcastro@salud-interactiva.com.mx" xr:uid="{07A9FA01-537D-43F7-AC04-CD326B68A11C}"/>
+    <hyperlink ref="E4" r:id="rId3" display="mailto:lhernandez@salud-interactiva.com.mx" xr:uid="{20312DC5-6E04-4B10-8467-EC57ED5C6CDD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor email templates: update HTML structure, add new images, and remove obsolete files for VRIM
</commit_message>
<xml_diff>
--- a/PruebasCorreos.xlsx
+++ b/PruebasCorreos.xlsx
@@ -1,23 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Desktop\FarmaLeal-Mailing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roberto Monjardin\Desktop\Salud Interactiva\projects\mailing-salud-interactiva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F55B03A6-323F-4D0C-9567-518287B86CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{402CEBB4-4408-4BF8-AB9C-F7F2FFCA091B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{B3DB81C5-9EF5-45C7-8B63-AD43FCE30ABD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B3DB81C5-9EF5-45C7-8B63-AD43FCE30ABD}"/>
   </bookViews>
   <sheets>
     <sheet name="DETALLE" sheetId="4" r:id="rId1"/>
     <sheet name="Hoja1" sheetId="5" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DETALLE!$E$1:$J$5</definedName>
+    <definedName name="Estado">[1]Catálogos!$AP$2:$AP$33</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="45">
   <si>
     <t>UN</t>
   </si>
@@ -114,40 +118,65 @@
     <t>christian.lepe@farmaleal.com.mx</t>
   </si>
   <si>
-    <t>rmonjardin@salud-interactiva.com.mx</t>
-  </si>
-  <si>
-    <t>Producto</t>
-  </si>
-  <si>
-    <t>NumeroTarjeta</t>
-  </si>
-  <si>
-    <t>NomCompleto</t>
-  </si>
-  <si>
-    <t>VIG</t>
-  </si>
-  <si>
-    <t>EtiquetaLogistica02</t>
-  </si>
-  <si>
-    <t>EtiquetaLogistica03</t>
-  </si>
-  <si>
     <t>BLACK VRIM DIGITAL- GENERICO</t>
   </si>
   <si>
-    <t>'1122052600028094</t>
-  </si>
-  <si>
-    <t>'14/MAY/2027</t>
-  </si>
-  <si>
-    <t>'1122052600028096</t>
-  </si>
-  <si>
-    <t>Christian Lepe Cruz</t>
+    <t>Nombre Oficina</t>
+  </si>
+  <si>
+    <t>Fecha de Cuenta
+dd-mmm-aa</t>
+  </si>
+  <si>
+    <t>Folio Solicitud</t>
+  </si>
+  <si>
+    <t>Número de Tarjeta</t>
+  </si>
+  <si>
+    <t>Nombre Completo</t>
+  </si>
+  <si>
+    <t>CODIGO PRODUCTO</t>
+  </si>
+  <si>
+    <t>PRODUCTO</t>
+  </si>
+  <si>
+    <t>VIGENCIA</t>
+  </si>
+  <si>
+    <t>SUC. D VIVEROS (CDMX)</t>
+  </si>
+  <si>
+    <t>TYS995006000050091</t>
+  </si>
+  <si>
+    <t>1122062600028847</t>
+  </si>
+  <si>
+    <t>DI61</t>
+  </si>
+  <si>
+    <t>1122062600028849</t>
+  </si>
+  <si>
+    <t>ROBERTO EDGAR MONJARDIN ALVARDO</t>
+  </si>
+  <si>
+    <t>DI62</t>
+  </si>
+  <si>
+    <t>DI63</t>
+  </si>
+  <si>
+    <t>MARICELA CASTRO</t>
+  </si>
+  <si>
+    <t>mcastro@salud-interactiva.com.mx</t>
+  </si>
+  <si>
+    <t>CHRISTIAN LEPE CRUZ</t>
   </si>
   <si>
     <t>clepe@salud-interactiva.com.mx</t>
@@ -160,7 +189,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -203,8 +232,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -217,8 +263,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="57"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="53"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="42"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -227,12 +291,44 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color auto="1"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -244,7 +340,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1"/>
@@ -259,9 +355,51 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="5" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -293,6 +431,243 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Acceso"/>
+      <sheetName val="CuentaExpress"/>
+      <sheetName val="Recluta"/>
+      <sheetName val="MatrizProductos"/>
+      <sheetName val="Productos &gt; Insumos"/>
+      <sheetName val="Matriz ArtJuegos"/>
+      <sheetName val="Matriz de Insumos"/>
+      <sheetName val="Insumos Totales"/>
+      <sheetName val="Catálogos"/>
+      <sheetName val="Afiliados"/>
+      <sheetName val="Validación Ventas"/>
+      <sheetName val="Etiquetas"/>
+      <sheetName val="Reporte Emisión"/>
+      <sheetName val="GanaMas"/>
+      <sheetName val="BD SAC"/>
+      <sheetName val="frCuenta"/>
+      <sheetName val="Reporte de Ventas"/>
+      <sheetName val="Acumulado"/>
+      <sheetName val="Hoja6"/>
+      <sheetName val="Asesores"/>
+      <sheetName val="VENTA DIGITAL"/>
+      <sheetName val="Hoja2"/>
+      <sheetName val="Acumulado de ventas Dig"/>
+      <sheetName val="Ventas Dig PG"/>
+      <sheetName val="Ventas Digitales Ac Inbursa"/>
+      <sheetName val="Ventas Digitales Ac Vrim"/>
+      <sheetName val="Hoja1"/>
+      <sheetName val="Hoja3"/>
+      <sheetName val="Hoja4"/>
+      <sheetName val="Reporte de Ventas (2)"/>
+      <sheetName val="Hoja5"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8">
+        <row r="2">
+          <cell r="B2" t="str">
+            <v>CH01</v>
+          </cell>
+          <cell r="AP2" t="str">
+            <v>AGUASCALIENTES</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="AP3" t="str">
+            <v>BAJA CALIFORNIA</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="AP4" t="str">
+            <v>BAJA CALIFORNIA SUR</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="AP5" t="str">
+            <v>CAMPECHE</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="AP6" t="str">
+            <v>COAHUILA</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="AP7" t="str">
+            <v>COLIMA</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="AP8" t="str">
+            <v>CHIAPAS</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="AP9" t="str">
+            <v>CHIHUAHUA</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="AP10" t="str">
+            <v>DISTRITO FEDERAL</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="AP11" t="str">
+            <v>DURANGO</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="AP12" t="str">
+            <v>ESTADO DE MEXICO</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="AP13" t="str">
+            <v>GUANAJUATO</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="AP14" t="str">
+            <v>GUERRERO</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="AP15" t="str">
+            <v>HIDALGO</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="AP16" t="str">
+            <v>JALISCO</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="AP17" t="str">
+            <v>MICHOACAN</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="AP18" t="str">
+            <v>MORELOS</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="AP19" t="str">
+            <v>NAYARIT</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="AP20" t="str">
+            <v>NUEVO LEON</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="AP21" t="str">
+            <v>OAXACA</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="AP22" t="str">
+            <v>PUEBLA</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="AP23" t="str">
+            <v>QUERETARO</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="AP24" t="str">
+            <v>QUINTANA ROO</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="AP25" t="str">
+            <v>SAN LUIS POTOSI</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="AP26" t="str">
+            <v>SINALOA</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="AP27" t="str">
+            <v>SONORA</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="AP28" t="str">
+            <v>TABASCO</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="AP29" t="str">
+            <v>TAMAULIPAS</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="AP30" t="str">
+            <v>TLAXCALA</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="AP31" t="str">
+            <v>VERACRUZ</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="AP32" t="str">
+            <v>YUCATAN</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="AP33" t="str">
+            <v>ZACATECAS</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+      <sheetData sheetId="25"/>
+      <sheetData sheetId="26"/>
+      <sheetData sheetId="27"/>
+      <sheetData sheetId="28"/>
+      <sheetData sheetId="29"/>
+      <sheetData sheetId="30"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -885,7 +1260,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7100985-58AA-4CEE-9961-6E7E20BF57C2}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="37.140625" bestFit="1" customWidth="1"/>
@@ -895,117 +1270,167 @@
     <col min="6" max="6" width="41.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="10" t="s">
         <v>30</v>
       </c>
+      <c r="H1" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="10" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="16">
+        <v>46198</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="20">
+        <v>46563</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="16">
+        <v>46198</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F3" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="20">
+        <v>46563</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="11" t="s">
+      <c r="B4" s="16">
+        <v>46199</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="17" t="s">
         <v>24</v>
       </c>
+      <c r="I4" s="20">
+        <v>46564</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="16">
+        <v>46200</v>
+      </c>
+      <c r="C5" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>17</v>
+      <c r="D5" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="20">
+        <v>46565</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D10" s="9"/>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D9" s="9"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E5" xr:uid="{6C4833E7-8091-44BE-92F0-2DAC0B7402B5}">
+      <formula1>Estado</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="mailto:rmonjardin@salud-interactiva.com.mx" xr:uid="{BE9F2FF6-456F-4E2B-A0C0-BD76E4E06139}"/>
-    <hyperlink ref="F3" r:id="rId2" xr:uid="{091242AC-0F01-4ACA-8F19-964AD4F5C500}"/>
-    <hyperlink ref="F4" r:id="rId3" xr:uid="{688216C2-7797-4EEC-9184-3CB51A47873F}"/>
-    <hyperlink ref="F5" r:id="rId4" xr:uid="{A8FD61FC-4A75-44A7-BEE5-AD712FBB5B75}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{028D01FE-D171-4FA3-B6CA-6E6E13FACB2E}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{BFBABFEC-3D50-4EFD-AD17-24D251590BA0}"/>
+    <hyperlink ref="F5" r:id="rId3" xr:uid="{38ADAB76-D781-4983-8228-BF8485206627}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Enhance date handling: add date formatting functions and update vigencia processing in email logic
</commit_message>
<xml_diff>
--- a/PruebasCorreos.xlsx
+++ b/PruebasCorreos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roberto Monjardin\Desktop\Salud Interactiva\projects\mailing-salud-interactiva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{402CEBB4-4408-4BF8-AB9C-F7F2FFCA091B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B554AE0B-C3D1-4B18-9622-E81073B8F35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B3DB81C5-9EF5-45C7-8B63-AD43FCE30ABD}"/>
+    <workbookView xWindow="22932" yWindow="-156" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B3DB81C5-9EF5-45C7-8B63-AD43FCE30ABD}"/>
   </bookViews>
   <sheets>
     <sheet name="DETALLE" sheetId="4" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
   <si>
     <t>UN</t>
   </si>
@@ -162,24 +162,6 @@
   </si>
   <si>
     <t>ROBERTO EDGAR MONJARDIN ALVARDO</t>
-  </si>
-  <si>
-    <t>DI62</t>
-  </si>
-  <si>
-    <t>DI63</t>
-  </si>
-  <si>
-    <t>MARICELA CASTRO</t>
-  </si>
-  <si>
-    <t>mcastro@salud-interactiva.com.mx</t>
-  </si>
-  <si>
-    <t>CHRISTIAN LEPE CRUZ</t>
-  </si>
-  <si>
-    <t>clepe@salud-interactiva.com.mx</t>
   </si>
 </sst>
 </file>
@@ -1358,62 +1340,26 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="16">
-        <v>46199</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="20">
-        <v>46564</v>
-      </c>
+      <c r="A4" s="15"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="20"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="16">
-        <v>46200</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="I5" s="20">
-        <v>46565</v>
-      </c>
+      <c r="A5" s="15"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="20"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D9" s="9"/>
@@ -1428,9 +1374,8 @@
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{028D01FE-D171-4FA3-B6CA-6E6E13FACB2E}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{BFBABFEC-3D50-4EFD-AD17-24D251590BA0}"/>
-    <hyperlink ref="F5" r:id="rId3" xr:uid="{38ADAB76-D781-4983-8228-BF8485206627}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>